<commit_message>
Changes in Timesheet flow
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ArjunO360\O360-AI1\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajesh.ganesh\OneDrive - Speridian Technologies\Desktop\Automation\O360-AI1\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F552B83-7D55-4E60-AA6E-CF163A57A813}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7245" tabRatio="784" xr2:uid="{37B91979-A2CD-4275-8B46-28CAE73357A2}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7245" tabRatio="784" firstSheet="35" activeTab="40"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="54" r:id="rId1"/>
@@ -53,8 +52,9 @@
     <sheet name="Timesheet_Approvals" sheetId="45" r:id="rId38"/>
     <sheet name="TimeSheeEditDelete" sheetId="46" r:id="rId39"/>
     <sheet name="TimesheetOnBehalf" sheetId="47" r:id="rId40"/>
+    <sheet name="TimeSheetNew" sheetId="55" r:id="rId41"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="447">
   <si>
     <t>Run</t>
   </si>
@@ -1137,18 +1137,6 @@
     <t>May</t>
   </si>
   <si>
-    <t>May 18 - May 24</t>
-  </si>
-  <si>
-    <t>Sep</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1 </t>
-  </si>
-  <si>
-    <t>Swiss solutions inc</t>
-  </si>
-  <si>
     <t>Subject</t>
   </si>
   <si>
@@ -1381,12 +1369,48 @@
   </si>
   <si>
     <t>SPIND/O360/5089</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MAY 18 - MAY 24 </t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>range</t>
+  </si>
+  <si>
+    <t>Deployment/ Prod Cutover</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> June </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> JUN 01 - JUN 07 </t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>Mario.Noronha</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>O360@uaL!tY2O2twO</t>
+  </si>
+  <si>
+    <t>empName</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1531,7 +1555,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1663,6 +1687,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1977,7 +2003,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3618E37C-E82D-41F4-A0F6-14F2CE1C7F19}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1986,7 +2012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4CBCCBB-F620-4A1E-BF48-EA55E11F2AC6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AM2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2267,7 +2293,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71A94568-BE7D-4A57-AE37-C45034A52044}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2310,7 +2336,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDFDCC8D-039F-437D-A845-22D1EF423E12}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2356,14 +2382,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{8EFBC8F0-A848-41E5-BE64-C210D89A31CA}"/>
+    <hyperlink ref="D2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70ED1544-2BE3-4FC2-826F-03DF821EF92D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2406,7 +2432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B6B0AE9-A7B4-47F8-8613-52E7DBD9E269}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2442,7 +2468,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFD0D49B-4275-4C29-A7E4-3E5D2E2F9AC6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AN2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2651,7 +2677,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98277668-9C38-45A0-81A5-4103268AE99B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2728,7 +2754,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B26AF835-F3DC-4258-B7E9-8A704E59D479}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="21.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2797,7 +2823,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640F365E-94FE-4AC2-B5FD-37792E4BEBBE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AO2"/>
   <sheetFormatPr defaultColWidth="24.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2931,7 +2957,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C20F9C3-2077-46DF-BDF9-91D3A9296BF6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2988,7 +3014,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C05CB830-F643-4561-AC36-C2A46C3A1D52}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3015,62 +3041,62 @@
         <v>277</v>
       </c>
       <c r="D1" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="H1" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="I1" s="10" t="s">
         <v>362</v>
       </c>
-      <c r="F1" s="10" t="s">
-        <v>363</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>364</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>365</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>366</v>
-      </c>
       <c r="J1" s="12" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="J2" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -3080,7 +3106,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26032F91-1D32-41C8-80B5-14F121CB54B9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AR4"/>
   <sheetFormatPr defaultColWidth="24.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3253,7 +3279,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEB7CED6-2F35-4F60-8CB2-DEC660DA37B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AR6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3483,7 +3509,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C2F894F-4DFC-4FBB-B719-9794E831E694}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AQ2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3680,7 +3706,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{214CB241-6E87-4836-A252-56ABB1392CCF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3753,7 +3779,7 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C35003D-32FF-4C4E-B8D9-01131ECA7595}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3812,7 +3838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{295F87F1-5A5B-4876-8D59-558CC8D6B386}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="12.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3870,7 +3896,7 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{079E8DE2-777B-41A3-A3B2-D3A654D4814A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:W2"/>
   <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3992,7 +4018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97C9AFBD-E4D6-4804-9B2B-3F6869F8ABB2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultColWidth="11.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4058,7 +4084,7 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{001E4462-9A8A-44AF-8790-6421B6761FA3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U2"/>
   <sheetFormatPr defaultColWidth="47.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4196,7 +4222,7 @@
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C28F220E-131D-4310-9F23-98983252B9E2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4253,7 +4279,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B18F116-67D9-4FE1-A623-E49CFCDC1863}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4273,38 +4299,38 @@
         <v>277</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C3" s="13" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -4313,7 +4339,7 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B1AA0AA-5B10-429D-A29E-0FC5EF10B185}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4398,7 +4424,7 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62344A48-69E5-43B8-9D14-1FAC502B49A4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4456,7 +4482,7 @@
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9FF69B3-FB8A-4104-AD10-C989AE02930E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4504,7 +4530,7 @@
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA470D58-E3E5-4753-9210-1D5B01DBCD6E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4553,7 +4579,7 @@
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3798E0BB-1226-41F0-BA00-FA57325FB1DF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4601,7 +4627,7 @@
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E40C18C-8A6A-4622-AC55-0F628036286B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4652,7 +4678,7 @@
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{152573A1-17E3-4203-AC06-D8BFD7C45051}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AO2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4665,7 +4691,7 @@
     <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="22.5703125" customWidth="1"/>
-    <col min="13" max="13" width="21" customWidth="1"/>
+    <col min="13" max="13" width="21" style="58" customWidth="1"/>
     <col min="14" max="14" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="28" customWidth="1"/>
     <col min="16" max="16" width="20.7109375" customWidth="1"/>
@@ -4716,7 +4742,7 @@
       <c r="L1" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="M1" s="57" t="s">
         <v>92</v>
       </c>
       <c r="N1" s="10" t="s">
@@ -4803,8 +4829,8 @@
       <c r="L2" s="13" t="s">
         <v>356</v>
       </c>
-      <c r="M2" s="15" t="s">
-        <v>357</v>
+      <c r="M2" s="8" t="s">
+        <v>435</v>
       </c>
       <c r="N2" s="14" t="s">
         <v>111</v>
@@ -4813,16 +4839,16 @@
         <v>105</v>
       </c>
       <c r="P2" s="13" t="s">
-        <v>358</v>
-      </c>
-      <c r="Q2" s="16" t="s">
-        <v>359</v>
+        <v>356</v>
+      </c>
+      <c r="Q2" s="15">
+        <v>18</v>
       </c>
       <c r="R2" s="14">
         <v>1</v>
       </c>
-      <c r="S2" s="14" t="s">
-        <v>114</v>
+      <c r="S2" s="13" t="s">
+        <v>105</v>
       </c>
       <c r="T2" s="6" t="s">
         <v>115</v>
@@ -4830,8 +4856,8 @@
       <c r="U2" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="V2" s="14" t="s">
-        <v>360</v>
+      <c r="V2" s="13" t="s">
+        <v>105</v>
       </c>
       <c r="W2" s="17"/>
       <c r="X2" s="17"/>
@@ -4857,7 +4883,7 @@
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85ADAB9A-D995-469E-ADFD-83DA6A62D49E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4912,7 +4938,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="D2" s="18" t="s">
         <v>118</v>
@@ -4941,7 +4967,7 @@
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1FC31E0-B694-46DC-97A1-9877EF138762}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="21.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5016,7 +5042,7 @@
 </file>
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A5BF7F1-B735-432B-91CB-B3923E058B7F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AO2"/>
   <sheetFormatPr defaultColWidth="24.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -5093,7 +5119,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>128</v>
@@ -5111,10 +5137,10 @@
         <v>30</v>
       </c>
       <c r="I2" s="14">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="J2" s="14">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="K2" s="52" t="s">
         <v>282</v>
@@ -5154,7 +5180,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5D4DEE5-F39A-47A7-911C-C765D6D534B7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5182,80 +5208,80 @@
         <v>122</v>
       </c>
       <c r="E1" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="I1" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="J1" s="10" t="s">
         <v>362</v>
       </c>
-      <c r="G1" s="10" t="s">
-        <v>363</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>364</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>365</v>
-      </c>
-      <c r="J1" s="10" t="s">
+      <c r="K1" s="10" t="s">
         <v>366</v>
       </c>
-      <c r="K1" s="10" t="s">
-        <v>370</v>
-      </c>
       <c r="L1" s="10" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="D2" t="s">
+        <v>422</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>423</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>407</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>382</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="K2" s="13" t="s">
+        <v>424</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>425</v>
       </c>
-      <c r="D2" t="s">
+      <c r="M2" t="s">
         <v>426</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>427</v>
-      </c>
-      <c r="F2" s="23" t="s">
-        <v>410</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>411</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>385</v>
-      </c>
-      <c r="I2" s="23" t="s">
-        <v>386</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="K2" s="13" t="s">
-        <v>428</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="M2" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="D3" s="6" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="F3" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
     </row>
   </sheetData>
@@ -5264,7 +5290,7 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B9311BC-7647-48BC-960A-A6428A48C8D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5326,8 +5352,118 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.85546875" customWidth="1"/>
+    <col min="2" max="2" width="5.5703125" customWidth="1"/>
+    <col min="3" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" customWidth="1"/>
+    <col min="9" max="9" width="8" customWidth="1"/>
+    <col min="10" max="10" width="8.5703125" customWidth="1"/>
+    <col min="11" max="11" width="5.28515625" customWidth="1"/>
+    <col min="12" max="12" width="18.5703125" customWidth="1"/>
+    <col min="13" max="13" width="15.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>446</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>379</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>444</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>437</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+    </row>
+    <row r="2" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="H2" s="13" t="s">
+        <v>439</v>
+      </c>
+      <c r="I2" s="14">
+        <v>2025</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>440</v>
+      </c>
+      <c r="K2" s="14">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="M2" s="15"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="52"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{648EA32A-7D96-47D7-90E7-95212629AF91}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5352,106 +5488,106 @@
         <v>277</v>
       </c>
       <c r="D1" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>410</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>411</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>396</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>397</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="N1" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="O1" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="P1" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="Q1" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="R1" s="10" t="s">
         <v>362</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>414</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>364</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>370</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>415</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>400</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>401</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>402</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>361</v>
-      </c>
-      <c r="N1" s="10" t="s">
-        <v>362</v>
-      </c>
-      <c r="O1" s="10" t="s">
-        <v>363</v>
-      </c>
-      <c r="P1" s="10" t="s">
-        <v>364</v>
-      </c>
-      <c r="Q1" s="10" t="s">
-        <v>365</v>
-      </c>
-      <c r="R1" s="10" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="F2" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="J2" s="14"/>
       <c r="K2" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="L2" s="6"/>
       <c r="M2" s="14" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="N2" s="23" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="O2" s="14" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="P2" s="14" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="Q2" s="23" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="G3" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
     </row>
   </sheetData>
@@ -5461,7 +5597,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD8E4AC-A0D3-40DE-9448-FC9C9D66CEFB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5494,125 +5630,125 @@
         <v>277</v>
       </c>
       <c r="D1" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>396</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>397</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="N1" s="10" t="s">
+        <v>399</v>
+      </c>
+      <c r="O1" s="10" t="s">
+        <v>371</v>
+      </c>
+      <c r="P1" s="10" t="s">
+        <v>372</v>
+      </c>
+      <c r="Q1" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="R1" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="S1" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="T1" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="U1" s="10" t="s">
         <v>362</v>
       </c>
-      <c r="E1" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>364</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>370</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>372</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>400</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>401</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>402</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>373</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>374</v>
-      </c>
-      <c r="N1" s="10" t="s">
-        <v>403</v>
-      </c>
-      <c r="O1" s="10" t="s">
-        <v>375</v>
-      </c>
-      <c r="P1" s="10" t="s">
-        <v>376</v>
-      </c>
-      <c r="Q1" s="10" t="s">
-        <v>362</v>
-      </c>
-      <c r="R1" s="10" t="s">
-        <v>363</v>
-      </c>
-      <c r="S1" s="10" t="s">
-        <v>364</v>
-      </c>
-      <c r="T1" s="10" t="s">
-        <v>365</v>
-      </c>
-      <c r="U1" s="10" t="s">
-        <v>366</v>
-      </c>
       <c r="V1" s="10" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="I2" s="14" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="J2" s="23"/>
       <c r="K2" s="6"/>
       <c r="L2" s="5" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="M2" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="N2" t="s">
+        <v>404</v>
+      </c>
+      <c r="O2" s="21" t="s">
+        <v>392</v>
+      </c>
+      <c r="P2" s="21" t="s">
+        <v>405</v>
+      </c>
+      <c r="Q2" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="R2" s="14" t="s">
         <v>407</v>
       </c>
-      <c r="N2" t="s">
+      <c r="S2" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="T2" s="23" t="s">
+        <v>382</v>
+      </c>
+      <c r="U2" s="6" t="s">
         <v>408</v>
       </c>
-      <c r="O2" s="21" t="s">
-        <v>396</v>
-      </c>
-      <c r="P2" s="21" t="s">
+      <c r="V2" s="56" t="s">
         <v>409</v>
-      </c>
-      <c r="Q2" s="23" t="s">
-        <v>410</v>
-      </c>
-      <c r="R2" s="14" t="s">
-        <v>411</v>
-      </c>
-      <c r="S2" s="14" t="s">
-        <v>385</v>
-      </c>
-      <c r="T2" s="23" t="s">
-        <v>386</v>
-      </c>
-      <c r="U2" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="V2" s="56" t="s">
-        <v>413</v>
       </c>
     </row>
   </sheetData>
@@ -5622,7 +5758,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8A3AE85-FBFB-494B-AD4C-727F1C9B62D2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5657,129 +5793,129 @@
         <v>277</v>
       </c>
       <c r="D1" s="53" t="s">
+        <v>357</v>
+      </c>
+      <c r="E1" s="54" t="s">
+        <v>358</v>
+      </c>
+      <c r="F1" s="54" t="s">
+        <v>359</v>
+      </c>
+      <c r="G1" s="54" t="s">
+        <v>360</v>
+      </c>
+      <c r="H1" s="54" t="s">
         <v>361</v>
       </c>
-      <c r="E1" s="54" t="s">
+      <c r="I1" s="54" t="s">
         <v>362</v>
       </c>
-      <c r="F1" s="54" t="s">
+      <c r="J1" s="12" t="s">
         <v>363</v>
       </c>
-      <c r="G1" s="54" t="s">
+      <c r="K1" s="12" t="s">
         <v>364</v>
       </c>
-      <c r="H1" s="54" t="s">
+      <c r="L1" s="54" t="s">
         <v>365</v>
       </c>
-      <c r="I1" s="54" t="s">
+      <c r="M1" s="54" t="s">
         <v>366</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="N1" s="54" t="s">
         <v>367</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="O1" s="54" t="s">
         <v>368</v>
       </c>
-      <c r="L1" s="54" t="s">
+      <c r="P1" s="54" t="s">
         <v>369</v>
       </c>
-      <c r="M1" s="54" t="s">
+      <c r="Q1" s="54" t="s">
         <v>370</v>
       </c>
-      <c r="N1" s="54" t="s">
+      <c r="R1" s="54" t="s">
         <v>371</v>
       </c>
-      <c r="O1" s="54" t="s">
+      <c r="S1" s="54" t="s">
         <v>372</v>
       </c>
-      <c r="P1" s="54" t="s">
+      <c r="T1" s="10" t="s">
         <v>373</v>
       </c>
-      <c r="Q1" s="54" t="s">
+      <c r="U1" s="10" t="s">
         <v>374</v>
       </c>
-      <c r="R1" s="54" t="s">
+      <c r="V1" s="10" t="s">
         <v>375</v>
-      </c>
-      <c r="S1" s="54" t="s">
-        <v>376</v>
-      </c>
-      <c r="T1" s="10" t="s">
-        <v>377</v>
-      </c>
-      <c r="U1" s="10" t="s">
-        <v>378</v>
-      </c>
-      <c r="V1" s="10" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>379</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>380</v>
+      </c>
+      <c r="G2" s="14" t="s">
         <v>381</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="H2" s="14" t="s">
         <v>382</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="I2" s="23" t="s">
         <v>383</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="J2" s="23" t="s">
         <v>384</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="K2" t="s">
         <v>385</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="L2" s="23" t="s">
         <v>386</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="M2" s="23" t="s">
         <v>387</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="N2" s="6" t="s">
         <v>388</v>
       </c>
-      <c r="K2" t="s">
+      <c r="O2" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="L2" s="23" t="s">
+      <c r="P2" s="14" t="s">
         <v>390</v>
       </c>
-      <c r="M2" s="23" t="s">
+      <c r="Q2" s="14" t="s">
         <v>391</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="R2" s="21" t="s">
         <v>392</v>
       </c>
-      <c r="O2" s="14" t="s">
+      <c r="S2" s="21" t="s">
         <v>393</v>
       </c>
-      <c r="P2" s="14" t="s">
+      <c r="T2" s="23" t="s">
         <v>394</v>
-      </c>
-      <c r="Q2" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="R2" s="21" t="s">
-        <v>396</v>
-      </c>
-      <c r="S2" s="21" t="s">
-        <v>397</v>
-      </c>
-      <c r="T2" s="23" t="s">
-        <v>398</v>
       </c>
       <c r="U2" s="5">
         <v>1</v>
       </c>
       <c r="V2" s="55" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
     </row>
   </sheetData>
@@ -5789,7 +5925,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08530B9C-4267-4988-BE10-30D04D9192FB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AG2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6031,7 +6167,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" xr:uid="{0F15AA83-BB5A-4AC8-B4C6-1859D69B0A5D}"/>
+    <hyperlink ref="H2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -6039,7 +6175,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58A15975-1EF1-4541-8083-A56DE49427DB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AA2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
Latest Changes at 26th June 25
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajesh.ganesh\OneDrive - Speridian Technologies\Desktop\Automation\O360-AI1\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Automation NEw\Arjun All Automation scripts\Rajesh 3\O360-AI1\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B8DA5F7-D6CA-4777-BDAF-7315E4C71F5C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7245" tabRatio="784" firstSheet="36" activeTab="41"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7245" tabRatio="784" firstSheet="16" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="54" r:id="rId1"/>
@@ -65,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="475">
   <si>
     <t>Run</t>
   </si>
@@ -1390,9 +1391,6 @@
     <t xml:space="preserve"> June </t>
   </si>
   <si>
-    <t xml:space="preserve"> JUN 01 - JUN 07 </t>
-  </si>
-  <si>
     <t>day</t>
   </si>
   <si>
@@ -1484,12 +1482,21 @@
   </si>
   <si>
     <t>billVerificationUserName</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> JUN 08 - JUN 14 </t>
+  </si>
+  <si>
+    <t>TC_Expenses</t>
+  </si>
+  <si>
+    <t>JUL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2124,7 +2131,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -2133,7 +2140,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:AM2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2414,7 +2421,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2457,7 +2464,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2503,14 +2510,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2553,7 +2560,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2589,7 +2596,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:AN2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2798,7 +2805,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2875,7 +2882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="21.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2944,7 +2951,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:AO2"/>
   <sheetFormatPr defaultColWidth="24.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3078,7 +3085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3135,7 +3142,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3227,7 +3234,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:AR4"/>
   <sheetFormatPr defaultColWidth="24.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3319,19 +3326,19 @@
         <v>2025</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>150</v>
+        <v>474</v>
       </c>
       <c r="F2" s="22">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="G2" s="14">
         <v>2025</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>150</v>
+        <v>474</v>
       </c>
       <c r="I2" s="23">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="J2" t="s">
         <v>151</v>
@@ -3400,7 +3407,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:AR6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3630,7 +3637,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:AQ2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3827,7 +3834,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3900,7 +3907,7 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3959,7 +3966,7 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="12.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4017,7 +4024,7 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <dimension ref="A1:W2"/>
   <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4139,7 +4146,7 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultColWidth="11.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4205,7 +4212,7 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:U2"/>
   <sheetFormatPr defaultColWidth="47.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4343,7 +4350,7 @@
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4400,7 +4407,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4460,7 +4467,7 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4545,7 +4552,7 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4603,7 +4610,7 @@
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4651,7 +4658,7 @@
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4700,7 +4707,7 @@
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4748,7 +4755,7 @@
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4799,7 +4806,7 @@
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <dimension ref="A1:AO2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5004,7 +5011,7 @@
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5088,7 +5095,7 @@
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="21.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5163,7 +5170,7 @@
 </file>
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:AO2"/>
   <sheetFormatPr defaultColWidth="24.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -5301,7 +5308,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5411,7 +5418,7 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5474,7 +5481,7 @@
 </file>
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
   <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5502,13 +5509,13 @@
         <v>255</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E1" s="9" t="s">
         <v>379</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>83</v>
@@ -5523,7 +5530,7 @@
         <v>437</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="L1" s="10" t="s">
         <v>438</v>
@@ -5548,10 +5555,10 @@
         <v>125</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="G2" s="13" t="s">
         <v>181</v>
@@ -5566,10 +5573,10 @@
         <v>440</v>
       </c>
       <c r="K2" s="14">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>441</v>
+        <v>472</v>
       </c>
       <c r="M2" s="15"/>
       <c r="N2" s="14"/>
@@ -5584,7 +5591,7 @@
 </file>
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2900-000000000000}">
   <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5620,10 +5627,10 @@
         <v>255</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F1" s="9" t="s">
         <v>436</v>
@@ -5632,54 +5639,54 @@
         <v>437</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I1" s="10" t="s">
         <v>83</v>
       </c>
       <c r="J1" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="K1" s="10" t="s">
         <v>447</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="L1" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="M1" s="10" t="s">
         <v>449</v>
       </c>
-      <c r="M1" s="10" t="s">
-        <v>450</v>
-      </c>
       <c r="N1" s="12" t="s">
+        <v>453</v>
+      </c>
+      <c r="O1" s="12" t="s">
         <v>454</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="P1" s="12" t="s">
         <v>455</v>
       </c>
-      <c r="P1" s="12" t="s">
-        <v>456</v>
-      </c>
       <c r="Q1" s="12" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="R1" s="12" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="S1" s="12" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="T1" s="12" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U1" s="12" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="V1" s="12" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="2" spans="1:22" s="8" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>104</v>
+        <v>473</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>2</v>
@@ -5688,7 +5695,7 @@
         <v>282</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>125</v>
@@ -5697,7 +5704,7 @@
         <v>2025</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="H2" s="13">
         <v>10</v>
@@ -5709,40 +5716,40 @@
         <v>201</v>
       </c>
       <c r="K2" s="13" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="L2" s="13">
         <v>122</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="N2" s="59" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="O2" s="61" t="s">
+        <v>458</v>
+      </c>
+      <c r="P2" s="6" t="s">
         <v>459</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="Q2" s="60" t="s">
         <v>460</v>
       </c>
-      <c r="Q2" s="60" t="s">
-        <v>461</v>
-      </c>
       <c r="R2" s="6" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="S2" s="8" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="T2" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U2" s="8" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="V2" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>
@@ -5751,7 +5758,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5885,7 +5892,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6046,7 +6053,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6213,7 +6220,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:AG2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6455,7 +6462,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -6463,7 +6470,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:AA2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>